<commit_message>
Actualiza calendario: agrega retiros de Monterrey (#121, #122) y Chihuahua (#3)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -8,23 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/17. CALENDARIO - EL VIVE - COMUNIDAD/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_89528FE70544D279036053753F009A56314D1768" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31F60562-0067-43E6-8ED6-AAA296880D8B}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_89528FE70544D279036053753F009A56314D1768" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD7FE047-9F77-47F1-95CC-6D43DFC0BEA3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendario" sheetId="1" r:id="rId1"/>
     <sheet name="Instrucciones" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Calendario!$A$1:$H$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Calendario!$A$1:$H$56</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="78">
   <si>
     <t>Mes</t>
   </si>
@@ -234,6 +234,30 @@
   </si>
   <si>
     <t>Domingo</t>
+  </si>
+  <si>
+    <t>24 – 26</t>
+  </si>
+  <si>
+    <t>Vie a Dom</t>
+  </si>
+  <si>
+    <t>Retiro #121 de Monterrey</t>
+  </si>
+  <si>
+    <t>Nos unimos todos en oración</t>
+  </si>
+  <si>
+    <t>31 – 2</t>
+  </si>
+  <si>
+    <t>Retiro #122 de Monterrey</t>
+  </si>
+  <si>
+    <t>4 – 6</t>
+  </si>
+  <si>
+    <t>Retiro #3 de Chihuahua</t>
   </si>
 </sst>
 </file>
@@ -628,7 +652,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -889,30 +913,32 @@
       <c r="A12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="2">
-        <v>20</v>
+      <c r="B12" s="2" t="s">
+        <v>70</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>9</v>
+        <v>71</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="3"/>
-      <c r="H12" s="2"/>
+        <v>72</v>
+      </c>
+      <c r="F12" s="2"/>
+      <c r="G12" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B13" s="2">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>9</v>
@@ -931,85 +957,89 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>25</v>
+        <v>17</v>
+      </c>
+      <c r="B14" s="2">
+        <v>27</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F14" s="2"/>
-      <c r="G14" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="3"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B15" s="2">
-        <v>11</v>
+      <c r="B15" s="2" t="s">
+        <v>74</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="F15" s="2"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="2"/>
+      <c r="G15" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="2">
-        <v>17</v>
+      <c r="B16" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="3"/>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="G16" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B17" s="2">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="3"/>
@@ -1020,7 +1050,7 @@
         <v>24</v>
       </c>
       <c r="B18" s="2">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>9</v>
@@ -1042,16 +1072,16 @@
         <v>24</v>
       </c>
       <c r="B19" s="2">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="3"/>
@@ -1062,53 +1092,49 @@
         <v>24</v>
       </c>
       <c r="B20" s="2">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>22</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="G20" s="3"/>
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B21" s="2">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>12</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="F21" s="2"/>
       <c r="G21" s="3"/>
       <c r="H21" s="2"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B22" s="2">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>15</v>
@@ -1117,7 +1143,7 @@
         <v>19</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>21</v>
@@ -1127,21 +1153,21 @@
       </c>
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="B23" s="2">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>12</v>
@@ -1153,42 +1179,48 @@
       <c r="A24" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B24" s="2">
-        <v>14</v>
+      <c r="B24" s="2" t="s">
+        <v>76</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>9</v>
+        <v>71</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="3"/>
-      <c r="H24" s="2"/>
+        <v>77</v>
+      </c>
+      <c r="F24" s="2"/>
+      <c r="G24" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B25" s="2">
+        <v>5</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="D25" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F25" s="2"/>
-      <c r="G25" s="3"/>
+        <v>36</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="H25" s="2"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1196,18 +1228,20 @@
         <v>35</v>
       </c>
       <c r="B26" s="2">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F26" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G26" s="3"/>
       <c r="H26" s="2"/>
     </row>
@@ -1216,7 +1250,7 @@
         <v>35</v>
       </c>
       <c r="B27" s="2">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>9</v>
@@ -1238,53 +1272,47 @@
         <v>35</v>
       </c>
       <c r="B28" s="2">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>22</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="F28" s="2"/>
+      <c r="G28" s="3"/>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B29" s="2">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>12</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="F29" s="2"/>
       <c r="G29" s="3"/>
       <c r="H29" s="2"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B30" s="2">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>9</v>
@@ -1301,43 +1329,45 @@
       <c r="G30" s="3"/>
       <c r="H30" s="2"/>
     </row>
-    <row r="31" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B31" s="2">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F31" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="G31" s="3" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B32" s="2">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>12</v>
@@ -1350,41 +1380,43 @@
         <v>38</v>
       </c>
       <c r="B33" s="2">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F33" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G33" s="3"/>
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B34" s="2">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G34" s="3"/>
+        <v>39</v>
+      </c>
+      <c r="F34" s="2"/>
+      <c r="G34" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="H34" s="2"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -1392,18 +1424,20 @@
         <v>38</v>
       </c>
       <c r="B35" s="2">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F35" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G35" s="3"/>
       <c r="H35" s="2"/>
     </row>
@@ -1412,40 +1446,36 @@
         <v>38</v>
       </c>
       <c r="B36" s="2">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>22</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="F36" s="2"/>
+      <c r="G36" s="3"/>
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B37" s="2">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>12</v>
@@ -1455,63 +1485,67 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B38" s="2">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>12</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="F38" s="2"/>
       <c r="G38" s="3"/>
       <c r="H38" s="2"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B39" s="2">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="F39" s="2"/>
-      <c r="G39" s="3"/>
+        <v>20</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B40" s="2">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F40" s="2"/>
+        <v>14</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G40" s="3"/>
       <c r="H40" s="2"/>
     </row>
@@ -1520,7 +1554,7 @@
         <v>42</v>
       </c>
       <c r="B41" s="2">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>9</v>
@@ -1542,23 +1576,19 @@
         <v>42</v>
       </c>
       <c r="B42" s="2">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>45</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="F42" s="2"/>
+      <c r="G42" s="3"/>
       <c r="H42" s="2"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -1566,38 +1596,36 @@
         <v>42</v>
       </c>
       <c r="B43" s="2">
+        <v>7</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="E43" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>12</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="F43" s="2"/>
       <c r="G43" s="3"/>
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B44" s="2">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F44" s="2" t="s">
         <v>12</v>
@@ -1610,19 +1638,23 @@
         <v>42</v>
       </c>
       <c r="B45" s="2">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F45" s="2"/>
-      <c r="G45" s="3"/>
+        <v>44</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>45</v>
+      </c>
       <c r="H45" s="2"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -1630,7 +1662,7 @@
         <v>42</v>
       </c>
       <c r="B46" s="2">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>9</v>
@@ -1647,65 +1679,67 @@
       <c r="G46" s="3"/>
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B47" s="2">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F47" s="2"/>
+        <v>14</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G47" s="3"/>
       <c r="H47" s="2"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B48" s="2">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>12</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="F48" s="2"/>
       <c r="G48" s="3"/>
       <c r="H48" s="2"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B49" s="2">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F49" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G49" s="3"/>
       <c r="H49" s="2"/>
     </row>
@@ -1714,16 +1748,16 @@
         <v>47</v>
       </c>
       <c r="B50" s="2">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="F50" s="2"/>
       <c r="G50" s="3"/>
@@ -1734,18 +1768,20 @@
         <v>47</v>
       </c>
       <c r="B51" s="2">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F51" s="2"/>
+        <v>11</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="G51" s="3"/>
       <c r="H51" s="2"/>
     </row>
@@ -1754,21 +1790,19 @@
         <v>47</v>
       </c>
       <c r="B52" s="2">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F52" s="2"/>
-      <c r="G52" s="3" t="s">
-        <v>53</v>
-      </c>
+      <c r="G52" s="3"/>
       <c r="H52" s="2"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
@@ -1776,32 +1810,97 @@
         <v>47</v>
       </c>
       <c r="B53" s="2">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>27</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="3"/>
       <c r="H53" s="2"/>
     </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B54" s="2">
+        <v>12</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F54" s="2"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="2"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B55" s="2">
+        <v>14</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F55" s="2"/>
+      <c r="G55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H55" s="2"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B56" s="2">
+        <v>17</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F56" s="2"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H53" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <dataValidations count="3">
-    <dataValidation type="list" sqref="A2:A53" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <autoFilter ref="A1:H56" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <dataValidations count="4">
+    <dataValidation type="list" sqref="A2:A56" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Junio,Julio,Agosto,Septiembre,Octubre,Noviembre,Diciembre"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="D2:D53" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="D2:D11 D13:D14 D16:D23 D25:D56" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Lunes de Junta,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2:H53" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H56" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Sí,No"</formula1>
+    </dataValidation>
+    <dataValidation type="list" sqref="D12 D15 D24" xr:uid="{8A516F92-DE95-4946-9290-67409ECA3E07}">
+      <formula1>"Junta de Consejo,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mueve el Retiro #122 de Monterrey a Julio (31 jul - 2 ago)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/17. CALENDARIO - EL VIVE - COMUNIDAD/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="11_89528FE70544D279036053753F009A56314D1768" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD7FE047-9F77-47F1-95CC-6D43DFC0BEA3}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_89528FE70544D279036053753F009A56314D1768" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DED364B-1EFD-485B-AFE3-D1DB686C1155}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Calendario" sheetId="1" r:id="rId1"/>
@@ -979,7 +979,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>74</v>

</xml_diff>

<commit_message>
Apostolado del 30 de junio: agrega lugar (Hospital General) y hora (7:30 p.m.)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e685dc9ab05c5d49/03. EZ PROJECT MANAGEMENT/06. CLAUDE CODE/17. CALENDARIO - EL VIVE - COMUNIDAD/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="11_89528FE70544D279036053753F009A56314D1768" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{942D476E-C4A1-46D0-BE38-D4B38F264F8D}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="11_89528FE70544D279036053753F009A56314D1768" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95E15833-BE20-4C3C-8705-85C262B8E3B2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="81">
   <si>
     <t>Mes</t>
   </si>
@@ -263,7 +263,10 @@
     <t xml:space="preserve">Lugar y Fecha exacta por definir </t>
   </si>
   <si>
-    <t>Lugar y Hora por definir</t>
+    <t>7:30 p.m.</t>
+  </si>
+  <si>
+    <t>Hospital General del Estado (Blvd. Colosio y Quintero Arce)</t>
   </si>
 </sst>
 </file>
@@ -667,7 +670,7 @@
     <col min="4" max="4" width="26" customWidth="1"/>
     <col min="5" max="5" width="48" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
+    <col min="7" max="7" width="55.140625" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
@@ -823,9 +826,11 @@
       <c r="E7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="2"/>
+      <c r="F7" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="G7" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H7" s="2"/>
     </row>
@@ -1886,16 +1891,16 @@
   </sheetData>
   <autoFilter ref="A1:H56" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <dataValidations count="4">
-    <dataValidation type="list" sqref="D16:D23 D25:D56 D14 D2:D4 D5:D12" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="D16:D23 D25:D56 D14 D2:D12" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Lunes de Junta,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="D13 D15 D24" xr:uid="{8A516F92-DE95-4946-9290-67409ECA3E07}">
       <formula1>"Junta de Consejo,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="A2:A4 A5:A56" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="A2:A56" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Junio,Julio,Agosto,Septiembre,Octubre,Noviembre,Diciembre"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2:H4 H5:H56" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H56" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fotos del Apostolado 1 de julio (4) + misas mensuales vuelven a domingo
- El Apostolado del 1 de julio ahora abre una galería "Ver fotos" con 4
  imágenes (la que ya existía + 3 nuevas); reemplaza el botón "Ver info"
- Misas mensuales movidas de sábado a domingo (Ago 30, Sep 6, Sep 27,
  Oct 25, Nov 15); regenerado desde el Excel

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -1238,11 +1238,11 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Sabado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H22" s="2" t="n"/>
@@ -1350,11 +1350,11 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1374,7 +1374,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Sabado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H25" s="2" t="n"/>
@@ -1548,11 +1548,11 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Sabado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H31" s="2" t="n"/>
@@ -1814,11 +1814,11 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Sabado</t>
+          <t>Domingo</t>
         </is>
       </c>
       <c r="H39" s="2" t="n"/>
@@ -2012,11 +2012,11 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -2393,7 +2393,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H56"/>
-  <dataValidations count="5">
+  <dataValidations count="4">
     <dataValidation sqref="D2:D12 D14 D16:D23 D25:D56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Lunes de Junta,Apostolado,Misa,Matrimonios · KIDS · Juntas,Económica,Especial"</formula1>
     </dataValidation>
@@ -2403,10 +2403,7 @@
     <dataValidation sqref="A2:A56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Junio,Julio,Agosto,Septiembre,Octubre,Noviembre,Diciembre"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sí,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H56 J2:J56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Apostolados mensuales ya con fecha definida (jul-dic)
29 jul, 19 ago, 23 sep, 14 oct (mie), 14 nov (sab) y 9 dic (mie).
Antes aparecian al final de cada mes como "fecha por definir";
ahora quedan en su dia, con la nota "Lugar por definir".

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -865,8 +865,14 @@
           <t>Julio</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
+      <c r="B11" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -880,7 +886,7 @@
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lugar y Fecha exacta por definir </t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H11" s="2" t="n"/>
@@ -1145,8 +1151,14 @@
           <t>Agosto</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
+      <c r="B19" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -1160,7 +1172,7 @@
       <c r="F19" s="2" t="n"/>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lugar y Fecha exacta por definir </t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H19" s="2" t="n"/>
@@ -1485,8 +1497,14 @@
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
+      <c r="B29" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -1500,7 +1518,7 @@
       <c r="F29" s="2" t="n"/>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lugar y Fecha exacta por definir </t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H29" s="2" t="n"/>
@@ -1721,8 +1739,14 @@
           <t>Octubre</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
+      <c r="B36" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -1736,7 +1760,7 @@
       <c r="F36" s="2" t="n"/>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lugar y Fecha exacta por definir </t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H36" s="2" t="n"/>
@@ -1949,8 +1973,14 @@
           <t>Noviembre</t>
         </is>
       </c>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="2" t="n"/>
+      <c r="B43" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Sáb</t>
+        </is>
+      </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -1964,7 +1994,7 @@
       <c r="F43" s="2" t="n"/>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lugar y Fecha exacta por definir </t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H43" s="2" t="n"/>
@@ -2181,8 +2211,14 @@
           <t>Diciembre</t>
         </is>
       </c>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
+      <c r="B50" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Mié</t>
+        </is>
+      </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Apostolado</t>
@@ -2196,7 +2232,7 @@
       <c r="F50" s="2" t="n"/>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lugar y Fecha exacta por definir </t>
+          <t>Lugar por definir</t>
         </is>
       </c>
       <c r="H50" s="2" t="n"/>

</xml_diff>

<commit_message>
Agosto: intercambio de fechas de dos juntas
- Matrimonios ÉL VIVE, KIDS y Juntas: 31 → 24 (lunes)
- Junta de Comunidad / INI: 24 → 31 (lunes)

Editado en el Excel (fuente) y regenerado con actualizar.py.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -1186,7 +1186,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
@@ -1288,7 +1288,7 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Septiembre: quita Misa de Niños (6 sep) y renombra la misa del 27 a «Misa Mensual - Misa de niños»
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/calendario-el-vive.xlsx
+++ b/datos/calendario-el-vive.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1362,33 +1362,29 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Misa de Niños</t>
+          <t>Junta de Comunidad / INI</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="n"/>
       <c r="H25" s="2" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="2" t="n"/>
@@ -1400,7 +1396,7 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
@@ -1434,28 +1430,24 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
+          <t>Kermés de la Parroquia La Resurrección</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n"/>
       <c r="G27" s="3" t="n"/>
       <c r="H27" s="2" t="n"/>
       <c r="I27" s="3" t="n"/>
@@ -1468,25 +1460,29 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Kermés de la Parroquia La Resurrección</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F28" s="2" t="n"/>
-      <c r="G28" s="3" t="n"/>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="2" t="n"/>
@@ -1498,29 +1494,29 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="n"/>
       <c r="H29" s="2" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="2" t="n"/>
@@ -1532,29 +1528,33 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
+          <t>Misa Mensual - Misa de niños</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="n"/>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="2" t="n"/>
@@ -1566,33 +1566,29 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="n"/>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="2" t="n"/>
@@ -1600,11 +1596,11 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Septiembre</t>
+          <t>Octubre</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
@@ -1613,12 +1609,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+          <t>Junta de Comunidad / INI</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1638,29 +1634,29 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G33" s="3" t="n"/>
+          <t>Primera limpieza de rancho con Comunidad de Iniciación 1</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Incluye un momento de convivencia, oración y encuentro en el rancho.</t>
+        </is>
+      </c>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="2" t="n"/>
@@ -1672,29 +1668,29 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Primera limpieza de rancho con Comunidad de Iniciación 1</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Incluye un momento de convivencia, oración y encuentro en el rancho.</t>
-        </is>
-      </c>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="n"/>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="2" t="n"/>
@@ -1706,29 +1702,29 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="n"/>
+          <t>Apostolado mensual</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="2" t="n"/>
@@ -1740,29 +1736,29 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="n"/>
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="2" t="n"/>
@@ -1774,28 +1770,24 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
+          <t>Actividad económica grande (Conferencias)</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n"/>
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="3" t="n"/>
@@ -1808,25 +1800,33 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Actividad económica grande (Conferencias)</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="3" t="n"/>
+          <t>Misa mensual</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Domingo</t>
+        </is>
+      </c>
       <c r="H38" s="2" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="2" t="n"/>
@@ -1838,33 +1838,29 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Domingo</t>
-        </is>
-      </c>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="n"/>
       <c r="H39" s="2" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="2" t="n"/>
@@ -1872,11 +1868,11 @@
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Octubre</t>
+          <t>Noviembre</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
@@ -1885,12 +1881,12 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
+          <t>Junta de Comunidad / INI</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1919,19 +1915,15 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
+          <t>Entrega de boletos de la Mega Rifa</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n"/>
       <c r="G41" s="3" t="n"/>
       <c r="H41" s="2" t="n"/>
       <c r="I41" s="3" t="n"/>
@@ -1944,25 +1936,29 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Entrega de boletos de la Mega Rifa</t>
+          <t>Apostolado mensual</t>
         </is>
       </c>
       <c r="F42" s="2" t="n"/>
-      <c r="G42" s="3" t="n"/>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H42" s="2" t="n"/>
       <c r="I42" s="3" t="n"/>
       <c r="J42" s="2" t="n"/>
@@ -1974,29 +1970,29 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="n"/>
       <c r="H43" s="2" t="n"/>
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="2" t="n"/>
@@ -2008,29 +2004,33 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Misa</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
+          <t>Misa mensual y convivencia con KIDS</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="n"/>
+          <t>5:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>(O apostolado con KIDS, por definir.)</t>
+        </is>
+      </c>
       <c r="H44" s="2" t="n"/>
       <c r="I44" s="3" t="n"/>
       <c r="J44" s="2" t="n"/>
@@ -2042,33 +2042,29 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Misa</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Misa mensual y convivencia con KIDS</t>
+          <t>Junta de Comunidad / INI</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>5:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>(O apostolado con KIDS, por definir.)</t>
-        </is>
-      </c>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="n"/>
       <c r="H45" s="2" t="n"/>
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="2" t="n"/>
@@ -2080,7 +2076,7 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
@@ -2089,12 +2085,12 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Matrimonios · KIDS · Juntas</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
+          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2114,28 +2110,24 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Matrimonios · KIDS · Juntas</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Matrimonios ÉL VIVE, KIDS y Juntas de Comunidad e Iniciación</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
+          <t>Limpieza de rancho</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n"/>
       <c r="G47" s="3" t="n"/>
       <c r="H47" s="2" t="n"/>
       <c r="I47" s="3" t="n"/>
@@ -2148,24 +2140,28 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Especial</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Limpieza de rancho</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="n"/>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
       <c r="G48" s="3" t="n"/>
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="3" t="n"/>
@@ -2174,33 +2170,33 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Noviembre</t>
+          <t>Diciembre</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mié</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Apostolado</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="n"/>
+          <t>Apostolado mensual</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Lugar por definir</t>
+        </is>
+      </c>
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="3" t="n"/>
       <c r="J49" s="2" t="n"/>
@@ -2212,29 +2208,29 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Mié</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Apostolado</t>
+          <t>Lunes de Junta</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Apostolado mensual</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="n"/>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Lugar por definir</t>
-        </is>
-      </c>
+          <t>Junta de Comunidad / INI</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>8:00 p.m.</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="n"/>
       <c r="H50" s="2" t="n"/>
       <c r="I50" s="3" t="n"/>
       <c r="J50" s="2" t="n"/>
@@ -2246,28 +2242,24 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Lunes de Junta</t>
+          <t>Económica</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Junta de Comunidad / INI</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>8:00 p.m.</t>
-        </is>
-      </c>
+          <t>Mega Rifa</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n"/>
       <c r="G51" s="3" t="n"/>
       <c r="H51" s="2" t="n"/>
       <c r="I51" s="3" t="n"/>
@@ -2280,21 +2272,21 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Vie</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Económica</t>
+          <t>Especial</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Mega Rifa</t>
+          <t>Peregrinación</t>
         </is>
       </c>
       <c r="F52" s="2" t="n"/>
@@ -2310,11 +2302,11 @@
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Vie</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -2324,7 +2316,7 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Peregrinación</t>
+          <t>Día de la Virgen, misa y Posada KIDS</t>
         </is>
       </c>
       <c r="F53" s="2" t="n"/>
@@ -2340,11 +2332,11 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Lun</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -2354,11 +2346,15 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Día de la Virgen, misa y Posada KIDS</t>
+          <t>Posada durante la junta</t>
         </is>
       </c>
       <c r="F54" s="2" t="n"/>
-      <c r="G54" s="3" t="n"/>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Última junta del mes de diciembre.</t>
+        </is>
+      </c>
       <c r="H54" s="2" t="n"/>
       <c r="I54" s="3" t="n"/>
       <c r="J54" s="2" t="n"/>
@@ -2370,11 +2366,11 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Lun</t>
+          <t>Jue</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -2384,48 +2380,14 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Posada durante la junta</t>
+          <t>Última Hora Santa del año</t>
         </is>
       </c>
       <c r="F55" s="2" t="n"/>
-      <c r="G55" s="3" t="inlineStr">
-        <is>
-          <t>Última junta del mes de diciembre.</t>
-        </is>
-      </c>
+      <c r="G55" s="3" t="n"/>
       <c r="H55" s="2" t="n"/>
       <c r="I55" s="3" t="n"/>
       <c r="J55" s="2" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>Diciembre</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>Jue</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>Especial</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>Última Hora Santa del año</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="n"/>
-      <c r="G56" s="3" t="n"/>
-      <c r="H56" s="2" t="n"/>
-      <c r="I56" s="3" t="n"/>
-      <c r="J56" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H56"/>

</xml_diff>